<commit_message>
feat(template): wire macro and industry feeds into Inputs sheet
Tag the relevant Inputs cells (rf, ERP, β, BAA, target op margin, sales-to-capital, terminal WACC, terminal ROIC) with Pipeline field paths so the populator overwrites the hardcoded defaults with extracted values when available. Templated defaults are preserved when extraction returns None — the populator distinguishes "no data, default kept" from "no data, cell empty" so analysts can read provenance off the cell comment.
</commit_message>
<xml_diff>
--- a/templates/valuation_template.xlsx
+++ b/templates/valuation_template.xlsx
@@ -138,11 +138,11 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -273,9 +273,49 @@
     <author>template</author>
   </authors>
   <commentList>
+    <comment ref="B3" authorId="0" shapeId="0">
+      <text>
+        <t>Pipeline field: macro.risk_free_rate</t>
+      </text>
+    </comment>
+    <comment ref="B4" authorId="0" shapeId="0">
+      <text>
+        <t>Pipeline field: industry.equity_risk_premium</t>
+      </text>
+    </comment>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Pipeline field: industry.levered_beta</t>
+      </text>
+    </comment>
+    <comment ref="B6" authorId="0" shapeId="0">
+      <text>
+        <t>Pipeline field: macro.baa_corporate_yield</t>
+      </text>
+    </comment>
     <comment ref="B8" authorId="0" shapeId="0">
       <text>
         <t>Pipeline field: tax.effective_rate</t>
+      </text>
+    </comment>
+    <comment ref="B12" authorId="0" shapeId="0">
+      <text>
+        <t>Pipeline field: industry.pretax_operating_margin</t>
+      </text>
+    </comment>
+    <comment ref="B14" authorId="0" shapeId="0">
+      <text>
+        <t>Pipeline field: industry.sales_to_capital</t>
+      </text>
+    </comment>
+    <comment ref="B18" authorId="0" shapeId="0">
+      <text>
+        <t>Pipeline field: industry.cost_of_capital</t>
+      </text>
+    </comment>
+    <comment ref="B19" authorId="0" shapeId="0">
+      <text>
+        <t>Pipeline field: industry.return_on_invested_capital</t>
       </text>
     </comment>
     <comment ref="B22" authorId="0" shapeId="0">
@@ -1375,7 +1415,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Tune to current yield as of valuation date.</t>
+          <t>Sourced from macro feed; override to lock.</t>
         </is>
       </c>
     </row>
@@ -1390,7 +1430,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Implied ERP; refresh quarterly from a standard source.</t>
+          <t>Sourced from industry feed (implied ERP); override to lock.</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1445,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Bottom-up: weighted avg of segment betas if multi-business.</t>
+          <t>Sourced from industry feed; bottom-up override is appropriate for multi-business issuers.</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1460,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>rf + spread implied by credit rating.</t>
+          <t>Sourced from macro feed (BAA corp yield); refine by credit rating.</t>
         </is>
       </c>
     </row>
@@ -1430,7 +1470,7 @@
           <t>Marginal tax rate</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="10" t="n">
         <v>0.25</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1445,7 +1485,7 @@
           <t>Effective tax rate (current)</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n"/>
+      <c r="B8" s="8" t="n"/>
       <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Provision / pre-tax income — pipeline pulls from filing.</t>
@@ -1468,12 +1508,12 @@
           <t>Compounded revenue growth, Y1-Y5</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="10" t="n">
         <v>0.08</v>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Glide path to terminal. Tune for thesis.</t>
+          <t>Glide path to terminal. Analyst thesis input.</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1528,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Year-10 EBIT margin; current margin is the start.</t>
+          <t>Sourced from industry feed; override for thesis upside/downside.</t>
         </is>
       </c>
     </row>
@@ -1518,7 +1558,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Reinvestment = ΔRevenue / S2C. Lower = more capital intensive.</t>
+          <t>Sourced from industry feed when available.</t>
         </is>
       </c>
     </row>
@@ -1538,12 +1578,12 @@
           <t>Terminal growth rate (perpetuity)</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n">
+      <c r="B17" s="10" t="n">
         <v>0.042</v>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Capped at risk-free rate.</t>
+          <t>Capped at risk-free rate. Analyst input.</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1598,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Converges to mature-firm WACC.</t>
+          <t>Sourced from industry feed (industry WACC); converges to mature-firm.</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1613,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Sustainable competitive return.</t>
+          <t>Sourced from industry feed; sustainable competitive return.</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2441,7 @@
           <t>Operating margin</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n"/>
+      <c r="B4" s="8" t="n"/>
       <c r="C4" s="22">
         <f>IFERROR(IF(1&gt;Inputs!B13,Inputs!B12,$B$4+((Inputs!B12-$B$4)/Inputs!B13)*1),"")</f>
         <v/>

</xml_diff>